<commit_message>
new complete Adblue manual
new complete Adblue manual to replace existing ones on the website
</commit_message>
<xml_diff>
--- a/Images for Markdown files database .xlsx
+++ b/Images for Markdown files database .xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trevor\Compac Industries\Compac - General\IT\ChatBot\Markdown-Manuals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1058868D-79DF-42E3-961D-C53D82C68E92}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5AA8729C-79CA-4954-82CA-5CE8F68172D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-1320" windowWidth="38640" windowHeight="21120" xr2:uid="{7323B22B-375C-41F7-91CD-F86C900FC6DE}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1150" uniqueCount="716">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="726">
   <si>
     <t xml:space="preserve">PCBs </t>
   </si>
@@ -2192,6 +2192,36 @@
   </si>
   <si>
     <t>6.1.5_GPIO_VeederRoot_EMR4_Pulser.png</t>
+  </si>
+  <si>
+    <t>AdBlue</t>
+  </si>
+  <si>
+    <t>19.1.1</t>
+  </si>
+  <si>
+    <t>19.1.1_AdBlue_hyd_module.png</t>
+  </si>
+  <si>
+    <t>19.2.1</t>
+  </si>
+  <si>
+    <t>19.3.1</t>
+  </si>
+  <si>
+    <t>19.4.1</t>
+  </si>
+  <si>
+    <t>19.4.1_AdBlue_ZVA_adblue_nozzle.png</t>
+  </si>
+  <si>
+    <t>19.3.1_AdBlue_solenoid_png</t>
+  </si>
+  <si>
+    <t>19.3.2_Adblue_piston_png</t>
+  </si>
+  <si>
+    <t>19.3.2</t>
   </si>
 </sst>
 </file>
@@ -2355,7 +2385,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="50">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2464,6 +2494,7 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7727,10 +7758,18 @@
       <c r="G412" s="5"/>
     </row>
     <row r="415" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A415" s="43"/>
-      <c r="B415" s="44"/>
-      <c r="C415" s="43"/>
-      <c r="D415" s="45"/>
+      <c r="A415" s="43">
+        <v>19</v>
+      </c>
+      <c r="B415" s="50" t="s">
+        <v>716</v>
+      </c>
+      <c r="C415" s="43" t="s">
+        <v>717</v>
+      </c>
+      <c r="D415" s="45" t="s">
+        <v>718</v>
+      </c>
       <c r="E415" s="43"/>
       <c r="F415" s="44"/>
       <c r="G415" s="44"/>
@@ -7768,7 +7807,9 @@
     <row r="418" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A418" s="43"/>
       <c r="B418" s="44"/>
-      <c r="C418" s="43"/>
+      <c r="C418" s="43" t="s">
+        <v>719</v>
+      </c>
       <c r="D418" s="44"/>
       <c r="E418" s="43"/>
       <c r="F418" s="44"/>
@@ -7820,8 +7861,12 @@
     <row r="422" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A422" s="43"/>
       <c r="B422" s="44"/>
-      <c r="C422" s="43"/>
-      <c r="D422" s="44"/>
+      <c r="C422" s="43" t="s">
+        <v>720</v>
+      </c>
+      <c r="D422" s="44" t="s">
+        <v>723</v>
+      </c>
       <c r="E422" s="43"/>
       <c r="F422" s="44"/>
       <c r="G422" s="44"/>
@@ -7833,8 +7878,12 @@
     <row r="423" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A423" s="43"/>
       <c r="B423" s="44"/>
-      <c r="C423" s="43"/>
-      <c r="D423" s="44"/>
+      <c r="C423" s="43" t="s">
+        <v>725</v>
+      </c>
+      <c r="D423" s="44" t="s">
+        <v>724</v>
+      </c>
       <c r="E423" s="43"/>
       <c r="F423" s="44"/>
       <c r="G423" s="44"/>
@@ -7872,8 +7921,12 @@
     <row r="426" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A426" s="43"/>
       <c r="B426" s="44"/>
-      <c r="C426" s="43"/>
-      <c r="D426" s="44"/>
+      <c r="C426" s="43" t="s">
+        <v>721</v>
+      </c>
+      <c r="D426" s="44" t="s">
+        <v>722</v>
+      </c>
       <c r="E426" s="43"/>
       <c r="F426" s="44"/>
       <c r="G426" s="44"/>

</xml_diff>

<commit_message>
new Gateway Lite manual
new Gateway Lite manual
</commit_message>
<xml_diff>
--- a/Images for Markdown files database .xlsx
+++ b/Images for Markdown files database .xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\trevor\Compac Industries\Compac - General\IT\ChatBot\Markdown-Manuals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD7C4140-385F-4A19-99B1-086C1C443892}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9EF3970-6AE4-4608-95C7-86A6CCF26CA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-38520" yWindow="-1320" windowWidth="38640" windowHeight="21120" xr2:uid="{7323B22B-375C-41F7-91CD-F86C900FC6DE}"/>
   </bookViews>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1380" uniqueCount="880">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1392" uniqueCount="892">
   <si>
     <t xml:space="preserve">PCBs </t>
   </si>
@@ -2685,6 +2685,42 @@
   </si>
   <si>
     <t>1.6.6_Terminals_MMR400_160S _ Avi_2x_C5K.png</t>
+  </si>
+  <si>
+    <t>12.16.5_ComfillV2_modem_LEDs.png</t>
+  </si>
+  <si>
+    <t>12.16.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12.16.6_Teltonika_router_LEDs.png </t>
+  </si>
+  <si>
+    <t>Gateway Lite</t>
+  </si>
+  <si>
+    <t>14.5.1</t>
+  </si>
+  <si>
+    <t>14.5.2</t>
+  </si>
+  <si>
+    <t>14.5.3</t>
+  </si>
+  <si>
+    <t>14.5.4</t>
+  </si>
+  <si>
+    <t>14.5.1_GW_Lite_dimensions.png</t>
+  </si>
+  <si>
+    <t>14.5.2_GW_Lite_mounting.png</t>
+  </si>
+  <si>
+    <t>15.5.3_GW_Lite_glands.png</t>
+  </si>
+  <si>
+    <t>14.5.4_GW_Lite_module.png</t>
   </si>
 </sst>
 </file>
@@ -3294,7 +3330,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2B533B56-556A-40A2-8D3F-E8E5A852019A}">
-  <dimension ref="A1:K460"/>
+  <dimension ref="A1:K465"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="11.26953125" style="1" customWidth="1"/>
@@ -7339,6 +7375,17 @@
       <c r="C333" s="1" t="s">
         <v>540</v>
       </c>
+      <c r="D333" t="s">
+        <v>880</v>
+      </c>
+    </row>
+    <row r="334" spans="2:4" x14ac:dyDescent="0.35">
+      <c r="C334" s="1" t="s">
+        <v>881</v>
+      </c>
+      <c r="D334" t="s">
+        <v>882</v>
+      </c>
     </row>
     <row r="336" spans="2:4" x14ac:dyDescent="0.35">
       <c r="B336" t="s">
@@ -7793,9 +7840,15 @@
     </row>
     <row r="381" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A381" s="4"/>
-      <c r="B381" s="5"/>
-      <c r="C381" s="4"/>
-      <c r="D381" s="5"/>
+      <c r="B381" s="5" t="s">
+        <v>883</v>
+      </c>
+      <c r="C381" s="4" t="s">
+        <v>884</v>
+      </c>
+      <c r="D381" s="5" t="s">
+        <v>888</v>
+      </c>
       <c r="E381" s="4"/>
       <c r="F381" s="5"/>
       <c r="G381" s="5"/>
@@ -7807,8 +7860,12 @@
     <row r="382" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A382" s="4"/>
       <c r="B382" s="5"/>
-      <c r="C382" s="4"/>
-      <c r="D382" s="5"/>
+      <c r="C382" s="4" t="s">
+        <v>885</v>
+      </c>
+      <c r="D382" s="5" t="s">
+        <v>889</v>
+      </c>
       <c r="E382" s="4"/>
       <c r="F382" s="5"/>
       <c r="G382" s="5"/>
@@ -7820,8 +7877,12 @@
     <row r="383" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A383" s="4"/>
       <c r="B383" s="5"/>
-      <c r="C383" s="4"/>
-      <c r="D383" s="5"/>
+      <c r="C383" s="4" t="s">
+        <v>886</v>
+      </c>
+      <c r="D383" s="5" t="s">
+        <v>890</v>
+      </c>
       <c r="E383" s="4"/>
       <c r="F383" s="5"/>
       <c r="G383" s="5"/>
@@ -7830,277 +7891,261 @@
       <c r="J383" s="5"/>
       <c r="K383" s="5"/>
     </row>
-    <row r="385" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C385" s="1" t="s">
+    <row r="384" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A384" s="4"/>
+      <c r="B384" s="5"/>
+      <c r="C384" s="4" t="s">
+        <v>887</v>
+      </c>
+      <c r="D384" s="5" t="s">
+        <v>891</v>
+      </c>
+      <c r="E384" s="4"/>
+      <c r="F384" s="5"/>
+      <c r="G384" s="5"/>
+      <c r="H384" s="5"/>
+      <c r="I384" s="5"/>
+      <c r="J384" s="5"/>
+      <c r="K384" s="5"/>
+    </row>
+    <row r="385" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A385" s="4"/>
+      <c r="B385" s="5"/>
+      <c r="C385" s="4"/>
+      <c r="D385" s="5"/>
+      <c r="E385" s="4"/>
+      <c r="F385" s="5"/>
+      <c r="G385" s="5"/>
+      <c r="H385" s="5"/>
+      <c r="I385" s="5"/>
+      <c r="J385" s="5"/>
+      <c r="K385" s="5"/>
+    </row>
+    <row r="386" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A386" s="4"/>
+      <c r="B386" s="5"/>
+      <c r="C386" s="4"/>
+      <c r="D386" s="5"/>
+      <c r="E386" s="4"/>
+      <c r="F386" s="5"/>
+      <c r="G386" s="5"/>
+      <c r="H386" s="5"/>
+      <c r="I386" s="5"/>
+      <c r="J386" s="5"/>
+      <c r="K386" s="5"/>
+    </row>
+    <row r="387" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A387" s="4"/>
+      <c r="B387" s="5"/>
+      <c r="C387" s="4"/>
+      <c r="D387" s="5"/>
+      <c r="E387" s="4"/>
+      <c r="F387" s="5"/>
+      <c r="G387" s="5"/>
+      <c r="H387" s="5"/>
+      <c r="I387" s="5"/>
+      <c r="J387" s="5"/>
+      <c r="K387" s="5"/>
+    </row>
+    <row r="388" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A388" s="4"/>
+      <c r="B388" s="5"/>
+      <c r="C388" s="4"/>
+      <c r="D388" s="5"/>
+      <c r="E388" s="4"/>
+      <c r="F388" s="5"/>
+      <c r="G388" s="5"/>
+      <c r="H388" s="5"/>
+      <c r="I388" s="5"/>
+      <c r="J388" s="5"/>
+      <c r="K388" s="5"/>
+    </row>
+    <row r="390" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C390" s="1" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="386" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C386" s="1" t="s">
+    <row r="391" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C391" s="1" t="s">
         <v>389</v>
       </c>
-      <c r="D386" t="s">
+      <c r="D391" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="387" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C387" s="1" t="s">
+    <row r="392" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C392" s="1" t="s">
         <v>391</v>
       </c>
-      <c r="D387" t="s">
+      <c r="D392" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="388" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C388" s="1" t="s">
+    <row r="393" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C393" s="1" t="s">
         <v>393</v>
       </c>
-      <c r="D388" t="s">
+      <c r="D393" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="389" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C389" s="1" t="s">
+    <row r="394" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C394" s="1" t="s">
         <v>395</v>
       </c>
-      <c r="D389" t="s">
+      <c r="D394" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="390" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C390" s="1" t="s">
+    <row r="395" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C395" s="1" t="s">
         <v>397</v>
       </c>
-      <c r="D390" t="s">
+      <c r="D395" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="391" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C391" s="1" t="s">
+    <row r="396" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C396" s="1" t="s">
         <v>399</v>
       </c>
-      <c r="D391" t="s">
+      <c r="D396" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="392" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C392" s="1" t="s">
+    <row r="397" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C397" s="1" t="s">
         <v>401</v>
       </c>
-      <c r="D392" t="s">
+      <c r="D397" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="393" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C393" s="1" t="s">
+    <row r="398" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C398" s="1" t="s">
         <v>403</v>
       </c>
-      <c r="D393" t="s">
+      <c r="D398" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="394" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C394" s="1" t="s">
+    <row r="399" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C399" s="1" t="s">
         <v>405</v>
       </c>
-      <c r="D394" t="s">
+      <c r="D399" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="395" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C395" s="1" t="s">
+    <row r="400" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C400" s="1" t="s">
         <v>407</v>
       </c>
-      <c r="D395" t="s">
+      <c r="D400" t="s">
         <v>404</v>
-      </c>
-    </row>
-    <row r="396" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C396" s="1" t="s">
-        <v>409</v>
-      </c>
-      <c r="D396" t="s">
-        <v>406</v>
-      </c>
-    </row>
-    <row r="397" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C397" s="1" t="s">
-        <v>411</v>
-      </c>
-      <c r="D397" t="s">
-        <v>408</v>
-      </c>
-    </row>
-    <row r="398" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C398" s="1" t="s">
-        <v>412</v>
-      </c>
-      <c r="D398" t="s">
-        <v>410</v>
-      </c>
-    </row>
-    <row r="399" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C399" s="1" t="s">
-        <v>414</v>
-      </c>
-      <c r="D399" t="s">
-        <v>413</v>
-      </c>
-    </row>
-    <row r="400" spans="3:4" x14ac:dyDescent="0.35">
-      <c r="C400" s="1" t="s">
-        <v>416</v>
-      </c>
-      <c r="D400" t="s">
-        <v>415</v>
       </c>
     </row>
     <row r="401" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C401" s="1" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="D401" t="s">
-        <v>417</v>
+        <v>406</v>
       </c>
     </row>
     <row r="402" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C402" s="1" t="s">
-        <v>420</v>
+        <v>411</v>
       </c>
       <c r="D402" t="s">
-        <v>419</v>
+        <v>408</v>
       </c>
     </row>
     <row r="403" spans="1:11" x14ac:dyDescent="0.35">
       <c r="C403" s="1" t="s">
+        <v>412</v>
+      </c>
+      <c r="D403" t="s">
+        <v>410</v>
+      </c>
+    </row>
+    <row r="404" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C404" s="1" t="s">
+        <v>414</v>
+      </c>
+      <c r="D404" t="s">
+        <v>413</v>
+      </c>
+    </row>
+    <row r="405" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C405" s="1" t="s">
+        <v>416</v>
+      </c>
+      <c r="D405" t="s">
+        <v>415</v>
+      </c>
+    </row>
+    <row r="406" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C406" s="1" t="s">
+        <v>418</v>
+      </c>
+      <c r="D406" t="s">
+        <v>417</v>
+      </c>
+    </row>
+    <row r="407" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C407" s="1" t="s">
+        <v>420</v>
+      </c>
+      <c r="D407" t="s">
+        <v>419</v>
+      </c>
+    </row>
+    <row r="408" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="C408" s="1" t="s">
         <v>422</v>
       </c>
-      <c r="D403" t="s">
+      <c r="D408" t="s">
         <v>421</v>
       </c>
     </row>
-    <row r="404" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="D404" t="s">
+    <row r="409" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="D409" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="405" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A405" s="26"/>
-      <c r="B405" s="25"/>
-      <c r="C405" s="26"/>
-      <c r="D405" s="25"/>
-      <c r="E405" s="26"/>
-      <c r="F405" s="25"/>
-      <c r="G405" s="25"/>
-      <c r="H405" s="25"/>
-      <c r="I405" s="25"/>
-      <c r="J405" s="25"/>
-      <c r="K405" s="25"/>
-    </row>
-    <row r="406" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A406" s="39">
+    <row r="410" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A410" s="26"/>
+      <c r="B410" s="25"/>
+      <c r="C410" s="26"/>
+      <c r="D410" s="25"/>
+      <c r="E410" s="26"/>
+      <c r="F410" s="25"/>
+      <c r="G410" s="25"/>
+      <c r="H410" s="25"/>
+      <c r="I410" s="25"/>
+      <c r="J410" s="25"/>
+      <c r="K410" s="25"/>
+    </row>
+    <row r="411" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A411" s="39">
         <v>16</v>
       </c>
-      <c r="B406" s="40" t="s">
+      <c r="B411" s="40" t="s">
         <v>385</v>
       </c>
-      <c r="C406" s="41" t="s">
+      <c r="C411" s="41" t="s">
         <v>337</v>
       </c>
-      <c r="D406" s="42" t="s">
+      <c r="D411" s="42" t="s">
         <v>349</v>
       </c>
-      <c r="E406" s="39" t="s">
+      <c r="E411" s="39" t="s">
         <v>565</v>
       </c>
-      <c r="F406" s="42" t="s">
+      <c r="F411" s="42" t="s">
         <v>385</v>
       </c>
-      <c r="G406" s="42"/>
-      <c r="H406" s="42"/>
-      <c r="I406" s="42"/>
-      <c r="J406" s="42"/>
-      <c r="K406" s="42"/>
-    </row>
-    <row r="407" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A407" s="39"/>
-      <c r="B407" s="42"/>
-      <c r="C407" s="41" t="s">
-        <v>338</v>
-      </c>
-      <c r="D407" s="42" t="s">
-        <v>350</v>
-      </c>
-      <c r="E407" s="39"/>
-      <c r="F407" s="42"/>
-      <c r="G407" s="42"/>
-      <c r="H407" s="42"/>
-      <c r="I407" s="42"/>
-      <c r="J407" s="42"/>
-      <c r="K407" s="42"/>
-    </row>
-    <row r="408" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A408" s="39"/>
-      <c r="B408" s="42"/>
-      <c r="C408" s="41" t="s">
-        <v>339</v>
-      </c>
-      <c r="D408" s="42" t="s">
-        <v>351</v>
-      </c>
-      <c r="E408" s="39"/>
-      <c r="F408" s="42"/>
-      <c r="G408" s="42"/>
-      <c r="H408" s="42"/>
-      <c r="I408" s="42"/>
-      <c r="J408" s="42"/>
-      <c r="K408" s="42"/>
-    </row>
-    <row r="409" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A409" s="39"/>
-      <c r="B409" s="42"/>
-      <c r="C409" s="41" t="s">
-        <v>340</v>
-      </c>
-      <c r="D409" s="42" t="s">
-        <v>352</v>
-      </c>
-      <c r="E409" s="39"/>
-      <c r="F409" s="42"/>
-      <c r="G409" s="42"/>
-      <c r="H409" s="42"/>
-      <c r="I409" s="42"/>
-      <c r="J409" s="42"/>
-      <c r="K409" s="42"/>
-    </row>
-    <row r="410" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A410" s="39"/>
-      <c r="B410" s="42"/>
-      <c r="C410" s="41" t="s">
-        <v>341</v>
-      </c>
-      <c r="D410" s="42" t="s">
-        <v>353</v>
-      </c>
-      <c r="E410" s="39"/>
-      <c r="F410" s="42"/>
-      <c r="G410" s="42"/>
-      <c r="H410" s="42"/>
-      <c r="I410" s="42"/>
-      <c r="J410" s="42"/>
-      <c r="K410" s="42"/>
-    </row>
-    <row r="411" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A411" s="39"/>
-      <c r="B411" s="42"/>
-      <c r="C411" s="41" t="s">
-        <v>342</v>
-      </c>
-      <c r="D411" s="42" t="s">
-        <v>354</v>
-      </c>
-      <c r="E411" s="39"/>
-      <c r="F411" s="42"/>
       <c r="G411" s="42"/>
       <c r="H411" s="42"/>
       <c r="I411" s="42"/>
@@ -8111,10 +8156,10 @@
       <c r="A412" s="39"/>
       <c r="B412" s="42"/>
       <c r="C412" s="41" t="s">
-        <v>343</v>
+        <v>338</v>
       </c>
       <c r="D412" s="42" t="s">
-        <v>355</v>
+        <v>350</v>
       </c>
       <c r="E412" s="39"/>
       <c r="F412" s="42"/>
@@ -8128,10 +8173,10 @@
       <c r="A413" s="39"/>
       <c r="B413" s="42"/>
       <c r="C413" s="41" t="s">
-        <v>344</v>
+        <v>339</v>
       </c>
       <c r="D413" s="42" t="s">
-        <v>356</v>
+        <v>351</v>
       </c>
       <c r="E413" s="39"/>
       <c r="F413" s="42"/>
@@ -8145,10 +8190,10 @@
       <c r="A414" s="39"/>
       <c r="B414" s="42"/>
       <c r="C414" s="41" t="s">
-        <v>345</v>
+        <v>340</v>
       </c>
       <c r="D414" s="42" t="s">
-        <v>357</v>
+        <v>352</v>
       </c>
       <c r="E414" s="39"/>
       <c r="F414" s="42"/>
@@ -8162,10 +8207,10 @@
       <c r="A415" s="39"/>
       <c r="B415" s="42"/>
       <c r="C415" s="41" t="s">
-        <v>346</v>
+        <v>341</v>
       </c>
       <c r="D415" s="42" t="s">
-        <v>359</v>
+        <v>353</v>
       </c>
       <c r="E415" s="39"/>
       <c r="F415" s="42"/>
@@ -8179,10 +8224,10 @@
       <c r="A416" s="39"/>
       <c r="B416" s="42"/>
       <c r="C416" s="41" t="s">
-        <v>347</v>
+        <v>342</v>
       </c>
       <c r="D416" s="42" t="s">
-        <v>358</v>
+        <v>354</v>
       </c>
       <c r="E416" s="39"/>
       <c r="F416" s="42"/>
@@ -8196,10 +8241,10 @@
       <c r="A417" s="39"/>
       <c r="B417" s="42"/>
       <c r="C417" s="41" t="s">
-        <v>348</v>
+        <v>343</v>
       </c>
       <c r="D417" s="42" t="s">
-        <v>360</v>
+        <v>355</v>
       </c>
       <c r="E417" s="39"/>
       <c r="F417" s="42"/>
@@ -8213,10 +8258,10 @@
       <c r="A418" s="39"/>
       <c r="B418" s="42"/>
       <c r="C418" s="41" t="s">
-        <v>372</v>
+        <v>344</v>
       </c>
       <c r="D418" s="42" t="s">
-        <v>361</v>
+        <v>356</v>
       </c>
       <c r="E418" s="39"/>
       <c r="F418" s="42"/>
@@ -8230,10 +8275,10 @@
       <c r="A419" s="39"/>
       <c r="B419" s="42"/>
       <c r="C419" s="41" t="s">
-        <v>373</v>
+        <v>345</v>
       </c>
       <c r="D419" s="42" t="s">
-        <v>362</v>
+        <v>357</v>
       </c>
       <c r="E419" s="39"/>
       <c r="F419" s="42"/>
@@ -8247,10 +8292,10 @@
       <c r="A420" s="39"/>
       <c r="B420" s="42"/>
       <c r="C420" s="41" t="s">
-        <v>374</v>
+        <v>346</v>
       </c>
       <c r="D420" s="42" t="s">
-        <v>363</v>
+        <v>359</v>
       </c>
       <c r="E420" s="39"/>
       <c r="F420" s="42"/>
@@ -8264,10 +8309,10 @@
       <c r="A421" s="39"/>
       <c r="B421" s="42"/>
       <c r="C421" s="41" t="s">
-        <v>375</v>
+        <v>347</v>
       </c>
       <c r="D421" s="42" t="s">
-        <v>364</v>
+        <v>358</v>
       </c>
       <c r="E421" s="39"/>
       <c r="F421" s="42"/>
@@ -8281,10 +8326,10 @@
       <c r="A422" s="39"/>
       <c r="B422" s="42"/>
       <c r="C422" s="41" t="s">
-        <v>376</v>
+        <v>348</v>
       </c>
       <c r="D422" s="42" t="s">
-        <v>365</v>
+        <v>360</v>
       </c>
       <c r="E422" s="39"/>
       <c r="F422" s="42"/>
@@ -8298,10 +8343,10 @@
       <c r="A423" s="39"/>
       <c r="B423" s="42"/>
       <c r="C423" s="41" t="s">
-        <v>377</v>
+        <v>372</v>
       </c>
       <c r="D423" s="42" t="s">
-        <v>366</v>
+        <v>361</v>
       </c>
       <c r="E423" s="39"/>
       <c r="F423" s="42"/>
@@ -8315,10 +8360,10 @@
       <c r="A424" s="39"/>
       <c r="B424" s="42"/>
       <c r="C424" s="41" t="s">
-        <v>378</v>
+        <v>373</v>
       </c>
       <c r="D424" s="42" t="s">
-        <v>367</v>
+        <v>362</v>
       </c>
       <c r="E424" s="39"/>
       <c r="F424" s="42"/>
@@ -8332,10 +8377,10 @@
       <c r="A425" s="39"/>
       <c r="B425" s="42"/>
       <c r="C425" s="41" t="s">
-        <v>379</v>
+        <v>374</v>
       </c>
       <c r="D425" s="42" t="s">
-        <v>368</v>
+        <v>363</v>
       </c>
       <c r="E425" s="39"/>
       <c r="F425" s="42"/>
@@ -8349,10 +8394,10 @@
       <c r="A426" s="39"/>
       <c r="B426" s="42"/>
       <c r="C426" s="41" t="s">
-        <v>380</v>
+        <v>375</v>
       </c>
       <c r="D426" s="42" t="s">
-        <v>369</v>
+        <v>364</v>
       </c>
       <c r="E426" s="39"/>
       <c r="F426" s="42"/>
@@ -8366,10 +8411,10 @@
       <c r="A427" s="39"/>
       <c r="B427" s="42"/>
       <c r="C427" s="41" t="s">
-        <v>381</v>
+        <v>376</v>
       </c>
       <c r="D427" s="42" t="s">
-        <v>370</v>
+        <v>365</v>
       </c>
       <c r="E427" s="39"/>
       <c r="F427" s="42"/>
@@ -8383,10 +8428,10 @@
       <c r="A428" s="39"/>
       <c r="B428" s="42"/>
       <c r="C428" s="41" t="s">
-        <v>382</v>
+        <v>377</v>
       </c>
       <c r="D428" s="42" t="s">
-        <v>371</v>
+        <v>366</v>
       </c>
       <c r="E428" s="39"/>
       <c r="F428" s="42"/>
@@ -8400,10 +8445,10 @@
       <c r="A429" s="39"/>
       <c r="B429" s="42"/>
       <c r="C429" s="41" t="s">
-        <v>383</v>
+        <v>378</v>
       </c>
       <c r="D429" s="42" t="s">
-        <v>384</v>
+        <v>367</v>
       </c>
       <c r="E429" s="39"/>
       <c r="F429" s="42"/>
@@ -8414,255 +8459,277 @@
       <c r="K429" s="42"/>
     </row>
     <row r="430" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A430" s="26"/>
-      <c r="B430" s="25"/>
-      <c r="C430" s="26"/>
-      <c r="D430" s="25"/>
-      <c r="E430" s="26"/>
-      <c r="F430" s="25"/>
-      <c r="G430" s="25"/>
-      <c r="H430" s="25"/>
-      <c r="I430" s="25"/>
-      <c r="J430" s="25"/>
-      <c r="K430" s="25"/>
+      <c r="A430" s="39"/>
+      <c r="B430" s="42"/>
+      <c r="C430" s="41" t="s">
+        <v>379</v>
+      </c>
+      <c r="D430" s="42" t="s">
+        <v>368</v>
+      </c>
+      <c r="E430" s="39"/>
+      <c r="F430" s="42"/>
+      <c r="G430" s="42"/>
+      <c r="H430" s="42"/>
+      <c r="I430" s="42"/>
+      <c r="J430" s="42"/>
+      <c r="K430" s="42"/>
     </row>
     <row r="431" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A431" s="32"/>
-      <c r="B431" s="33" t="s">
+      <c r="A431" s="39"/>
+      <c r="B431" s="42"/>
+      <c r="C431" s="41" t="s">
+        <v>380</v>
+      </c>
+      <c r="D431" s="42" t="s">
+        <v>369</v>
+      </c>
+      <c r="E431" s="39"/>
+      <c r="F431" s="42"/>
+      <c r="G431" s="42"/>
+      <c r="H431" s="42"/>
+      <c r="I431" s="42"/>
+      <c r="J431" s="42"/>
+      <c r="K431" s="42"/>
+    </row>
+    <row r="432" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A432" s="39"/>
+      <c r="B432" s="42"/>
+      <c r="C432" s="41" t="s">
+        <v>381</v>
+      </c>
+      <c r="D432" s="42" t="s">
+        <v>370</v>
+      </c>
+      <c r="E432" s="39"/>
+      <c r="F432" s="42"/>
+      <c r="G432" s="42"/>
+      <c r="H432" s="42"/>
+      <c r="I432" s="42"/>
+      <c r="J432" s="42"/>
+      <c r="K432" s="42"/>
+    </row>
+    <row r="433" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A433" s="39"/>
+      <c r="B433" s="42"/>
+      <c r="C433" s="41" t="s">
+        <v>382</v>
+      </c>
+      <c r="D433" s="42" t="s">
+        <v>371</v>
+      </c>
+      <c r="E433" s="39"/>
+      <c r="F433" s="42"/>
+      <c r="G433" s="42"/>
+      <c r="H433" s="42"/>
+      <c r="I433" s="42"/>
+      <c r="J433" s="42"/>
+      <c r="K433" s="42"/>
+    </row>
+    <row r="434" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A434" s="39"/>
+      <c r="B434" s="42"/>
+      <c r="C434" s="41" t="s">
+        <v>383</v>
+      </c>
+      <c r="D434" s="42" t="s">
+        <v>384</v>
+      </c>
+      <c r="E434" s="39"/>
+      <c r="F434" s="42"/>
+      <c r="G434" s="42"/>
+      <c r="H434" s="42"/>
+      <c r="I434" s="42"/>
+      <c r="J434" s="42"/>
+      <c r="K434" s="42"/>
+    </row>
+    <row r="435" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A435" s="26"/>
+      <c r="B435" s="25"/>
+      <c r="C435" s="26"/>
+      <c r="D435" s="25"/>
+      <c r="E435" s="26"/>
+      <c r="F435" s="25"/>
+      <c r="G435" s="25"/>
+      <c r="H435" s="25"/>
+      <c r="I435" s="25"/>
+      <c r="J435" s="25"/>
+      <c r="K435" s="25"/>
+    </row>
+    <row r="436" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A436" s="32"/>
+      <c r="B436" s="33" t="s">
         <v>424</v>
       </c>
-      <c r="C431" s="32" t="s">
+      <c r="C436" s="32" t="s">
         <v>425</v>
       </c>
-      <c r="D431" s="38" t="s">
+      <c r="D436" s="38" t="s">
         <v>426</v>
       </c>
-      <c r="E431" s="32"/>
-      <c r="F431" s="33"/>
-      <c r="G431" s="33"/>
-    </row>
-    <row r="432" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A432" s="4"/>
-      <c r="B432" s="5"/>
-      <c r="C432" s="4" t="s">
-        <v>427</v>
-      </c>
-      <c r="D432" s="18" t="s">
-        <v>428</v>
-      </c>
-      <c r="E432" s="4"/>
-      <c r="F432" s="5"/>
-      <c r="G432" s="5"/>
-    </row>
-    <row r="434" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A434" s="4"/>
-      <c r="B434" s="5" t="s">
-        <v>435</v>
-      </c>
-      <c r="C434" s="4" t="s">
-        <v>429</v>
-      </c>
-      <c r="D434" s="16" t="s">
-        <v>429</v>
-      </c>
-      <c r="E434" s="4"/>
-      <c r="F434" s="5"/>
-      <c r="G434" s="5"/>
-    </row>
-    <row r="435" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A435" s="4"/>
-      <c r="B435" s="5"/>
-      <c r="C435" s="4" t="s">
-        <v>430</v>
-      </c>
-      <c r="D435" s="16" t="s">
-        <v>430</v>
-      </c>
-      <c r="E435" s="4"/>
-      <c r="F435" s="5"/>
-      <c r="G435" s="5"/>
-    </row>
-    <row r="436" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A436" s="4"/>
-      <c r="B436" s="5"/>
-      <c r="C436" s="4" t="s">
-        <v>431</v>
-      </c>
-      <c r="D436" s="16" t="s">
-        <v>431</v>
-      </c>
-      <c r="E436" s="4"/>
-      <c r="F436" s="5"/>
-      <c r="G436" s="5"/>
-    </row>
-    <row r="437" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="E436" s="32"/>
+      <c r="F436" s="33"/>
+      <c r="G436" s="33"/>
+    </row>
+    <row r="437" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A437" s="4"/>
       <c r="B437" s="5"/>
       <c r="C437" s="4" t="s">
-        <v>432</v>
-      </c>
-      <c r="D437" s="16" t="s">
-        <v>432</v>
+        <v>427</v>
+      </c>
+      <c r="D437" s="18" t="s">
+        <v>428</v>
       </c>
       <c r="E437" s="4"/>
       <c r="F437" s="5"/>
       <c r="G437" s="5"/>
     </row>
-    <row r="438" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A438" s="4"/>
-      <c r="B438" s="5"/>
-      <c r="C438" s="4" t="s">
-        <v>433</v>
-      </c>
-      <c r="D438" s="16" t="s">
-        <v>433</v>
-      </c>
-      <c r="E438" s="4"/>
-      <c r="F438" s="5"/>
-      <c r="G438" s="5"/>
-    </row>
-    <row r="439" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="439" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A439" s="4"/>
-      <c r="B439" s="5"/>
-      <c r="C439" s="4"/>
-      <c r="D439" s="5"/>
+      <c r="B439" s="5" t="s">
+        <v>435</v>
+      </c>
+      <c r="C439" s="4" t="s">
+        <v>429</v>
+      </c>
+      <c r="D439" s="16" t="s">
+        <v>429</v>
+      </c>
       <c r="E439" s="4"/>
       <c r="F439" s="5"/>
       <c r="G439" s="5"/>
     </row>
-    <row r="440" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="440" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A440" s="4"/>
-      <c r="B440" s="5" t="s">
-        <v>436</v>
-      </c>
+      <c r="B440" s="5"/>
       <c r="C440" s="4" t="s">
-        <v>434</v>
+        <v>430</v>
       </c>
       <c r="D440" s="16" t="s">
-        <v>450</v>
+        <v>430</v>
       </c>
       <c r="E440" s="4"/>
-      <c r="F440" s="5" t="s">
-        <v>447</v>
-      </c>
+      <c r="F440" s="5"/>
       <c r="G440" s="5"/>
     </row>
-    <row r="441" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="441" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A441" s="4"/>
       <c r="B441" s="5"/>
       <c r="C441" s="4" t="s">
-        <v>437</v>
+        <v>431</v>
       </c>
       <c r="D441" s="16" t="s">
-        <v>451</v>
+        <v>431</v>
       </c>
       <c r="E441" s="4"/>
-      <c r="F441" s="5" t="s">
-        <v>448</v>
-      </c>
+      <c r="F441" s="5"/>
       <c r="G441" s="5"/>
     </row>
-    <row r="442" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="442" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A442" s="4"/>
       <c r="B442" s="5"/>
       <c r="C442" s="4" t="s">
-        <v>438</v>
+        <v>432</v>
       </c>
       <c r="D442" s="16" t="s">
-        <v>452</v>
+        <v>432</v>
       </c>
       <c r="E442" s="4"/>
-      <c r="F442" s="5" t="s">
-        <v>449</v>
-      </c>
+      <c r="F442" s="5"/>
       <c r="G442" s="5"/>
     </row>
-    <row r="443" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="443" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A443" s="4"/>
       <c r="B443" s="5"/>
       <c r="C443" s="4" t="s">
-        <v>439</v>
+        <v>433</v>
       </c>
       <c r="D443" s="16" t="s">
-        <v>454</v>
+        <v>433</v>
       </c>
       <c r="E443" s="4"/>
-      <c r="F443" s="5" t="s">
-        <v>453</v>
-      </c>
+      <c r="F443" s="5"/>
       <c r="G443" s="5"/>
     </row>
-    <row r="444" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="444" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A444" s="4"/>
       <c r="B444" s="5"/>
-      <c r="C444" s="4" t="s">
-        <v>440</v>
-      </c>
-      <c r="D444" s="16" t="s">
-        <v>440</v>
-      </c>
+      <c r="C444" s="4"/>
+      <c r="D444" s="5"/>
       <c r="E444" s="4"/>
       <c r="F444" s="5"/>
       <c r="G444" s="5"/>
     </row>
-    <row r="445" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="445" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A445" s="4"/>
-      <c r="B445" s="5"/>
-      <c r="C445" s="4"/>
-      <c r="D445" s="5"/>
+      <c r="B445" s="5" t="s">
+        <v>436</v>
+      </c>
+      <c r="C445" s="4" t="s">
+        <v>434</v>
+      </c>
+      <c r="D445" s="16" t="s">
+        <v>450</v>
+      </c>
       <c r="E445" s="4"/>
-      <c r="F445" s="5"/>
+      <c r="F445" s="5" t="s">
+        <v>447</v>
+      </c>
       <c r="G445" s="5"/>
     </row>
-    <row r="446" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="446" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A446" s="4"/>
-      <c r="B446" s="5" t="s">
-        <v>441</v>
-      </c>
+      <c r="B446" s="5"/>
       <c r="C446" s="4" t="s">
-        <v>442</v>
+        <v>437</v>
       </c>
       <c r="D446" s="16" t="s">
-        <v>442</v>
+        <v>451</v>
       </c>
       <c r="E446" s="4"/>
-      <c r="F446" s="5"/>
+      <c r="F446" s="5" t="s">
+        <v>448</v>
+      </c>
       <c r="G446" s="5"/>
     </row>
-    <row r="447" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="447" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A447" s="4"/>
       <c r="B447" s="5"/>
       <c r="C447" s="4" t="s">
-        <v>443</v>
+        <v>438</v>
       </c>
       <c r="D447" s="16" t="s">
-        <v>443</v>
+        <v>452</v>
       </c>
       <c r="E447" s="4"/>
-      <c r="F447" s="5"/>
+      <c r="F447" s="5" t="s">
+        <v>449</v>
+      </c>
       <c r="G447" s="5"/>
     </row>
-    <row r="448" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="448" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A448" s="4"/>
       <c r="B448" s="5"/>
       <c r="C448" s="4" t="s">
-        <v>444</v>
+        <v>439</v>
       </c>
       <c r="D448" s="16" t="s">
-        <v>444</v>
+        <v>454</v>
       </c>
       <c r="E448" s="4"/>
-      <c r="F448" s="5"/>
+      <c r="F448" s="5" t="s">
+        <v>453</v>
+      </c>
       <c r="G448" s="5"/>
     </row>
     <row r="449" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A449" s="4"/>
       <c r="B449" s="5"/>
       <c r="C449" s="4" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="D449" s="16" t="s">
-        <v>445</v>
+        <v>440</v>
       </c>
       <c r="E449" s="4"/>
       <c r="F449" s="5"/>
@@ -8671,111 +8738,91 @@
     <row r="450" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A450" s="4"/>
       <c r="B450" s="5"/>
-      <c r="C450" s="4" t="s">
-        <v>446</v>
-      </c>
-      <c r="D450" s="16" t="s">
-        <v>446</v>
-      </c>
+      <c r="C450" s="4"/>
+      <c r="D450" s="5"/>
       <c r="E450" s="4"/>
       <c r="F450" s="5"/>
       <c r="G450" s="5"/>
     </row>
+    <row r="451" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A451" s="4"/>
+      <c r="B451" s="5" t="s">
+        <v>441</v>
+      </c>
+      <c r="C451" s="4" t="s">
+        <v>442</v>
+      </c>
+      <c r="D451" s="16" t="s">
+        <v>442</v>
+      </c>
+      <c r="E451" s="4"/>
+      <c r="F451" s="5"/>
+      <c r="G451" s="5"/>
+    </row>
+    <row r="452" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A452" s="4"/>
+      <c r="B452" s="5"/>
+      <c r="C452" s="4" t="s">
+        <v>443</v>
+      </c>
+      <c r="D452" s="16" t="s">
+        <v>443</v>
+      </c>
+      <c r="E452" s="4"/>
+      <c r="F452" s="5"/>
+      <c r="G452" s="5"/>
+    </row>
     <row r="453" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A453" s="43">
+      <c r="A453" s="4"/>
+      <c r="B453" s="5"/>
+      <c r="C453" s="4" t="s">
+        <v>444</v>
+      </c>
+      <c r="D453" s="16" t="s">
+        <v>444</v>
+      </c>
+      <c r="E453" s="4"/>
+      <c r="F453" s="5"/>
+      <c r="G453" s="5"/>
+    </row>
+    <row r="454" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A454" s="4"/>
+      <c r="B454" s="5"/>
+      <c r="C454" s="4" t="s">
+        <v>445</v>
+      </c>
+      <c r="D454" s="16" t="s">
+        <v>445</v>
+      </c>
+      <c r="E454" s="4"/>
+      <c r="F454" s="5"/>
+      <c r="G454" s="5"/>
+    </row>
+    <row r="455" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A455" s="4"/>
+      <c r="B455" s="5"/>
+      <c r="C455" s="4" t="s">
+        <v>446</v>
+      </c>
+      <c r="D455" s="16" t="s">
+        <v>446</v>
+      </c>
+      <c r="E455" s="4"/>
+      <c r="F455" s="5"/>
+      <c r="G455" s="5"/>
+    </row>
+    <row r="458" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A458" s="43">
         <v>19</v>
       </c>
-      <c r="B453" s="50" t="s">
+      <c r="B458" s="50" t="s">
         <v>716</v>
       </c>
-      <c r="C453" s="43" t="s">
+      <c r="C458" s="43" t="s">
         <v>726</v>
       </c>
-      <c r="D453" s="44" t="s">
+      <c r="D458" s="44" t="s">
         <v>727</v>
-      </c>
-      <c r="E453" s="43"/>
-      <c r="F453" s="44"/>
-      <c r="G453" s="44"/>
-      <c r="H453" s="44"/>
-      <c r="I453" s="44"/>
-      <c r="J453" s="44"/>
-      <c r="K453" s="44"/>
-    </row>
-    <row r="454" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A454" s="43"/>
-      <c r="B454" s="44"/>
-      <c r="C454" s="43" t="s">
-        <v>717</v>
-      </c>
-      <c r="D454" s="45" t="s">
-        <v>718</v>
-      </c>
-      <c r="E454" s="43"/>
-      <c r="F454" s="44"/>
-      <c r="G454" s="44"/>
-      <c r="H454" s="44"/>
-      <c r="I454" s="44"/>
-      <c r="J454" s="44"/>
-      <c r="K454" s="44"/>
-    </row>
-    <row r="455" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A455" s="43"/>
-      <c r="B455" s="44"/>
-      <c r="C455" s="43" t="s">
-        <v>728</v>
-      </c>
-      <c r="D455" s="44" t="s">
-        <v>729</v>
-      </c>
-      <c r="E455" s="43"/>
-      <c r="F455" s="44"/>
-      <c r="G455" s="44"/>
-      <c r="H455" s="44"/>
-      <c r="I455" s="44"/>
-      <c r="J455" s="44"/>
-      <c r="K455" s="44"/>
-    </row>
-    <row r="456" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A456" s="43"/>
-      <c r="B456" s="44"/>
-      <c r="C456" s="43" t="s">
-        <v>719</v>
-      </c>
-      <c r="D456" s="44"/>
-      <c r="E456" s="43"/>
-      <c r="F456" s="44"/>
-      <c r="G456" s="44"/>
-      <c r="H456" s="44"/>
-      <c r="I456" s="44"/>
-      <c r="J456" s="44"/>
-      <c r="K456" s="44"/>
-    </row>
-    <row r="457" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A457" s="43"/>
-      <c r="B457" s="44"/>
-      <c r="C457" s="43" t="s">
-        <v>720</v>
-      </c>
-      <c r="D457" s="44" t="s">
-        <v>723</v>
-      </c>
-      <c r="E457" s="43"/>
-      <c r="F457" s="44"/>
-      <c r="G457" s="44"/>
-      <c r="H457" s="44"/>
-      <c r="I457" s="44"/>
-      <c r="J457" s="44"/>
-      <c r="K457" s="44"/>
-    </row>
-    <row r="458" spans="1:11" x14ac:dyDescent="0.35">
-      <c r="A458" s="43"/>
-      <c r="B458" s="44"/>
-      <c r="C458" s="43" t="s">
-        <v>725</v>
-      </c>
-      <c r="D458" s="44" t="s">
-        <v>724</v>
       </c>
       <c r="E458" s="43"/>
       <c r="F458" s="44"/>
@@ -8789,10 +8836,10 @@
       <c r="A459" s="43"/>
       <c r="B459" s="44"/>
       <c r="C459" s="43" t="s">
-        <v>721</v>
-      </c>
-      <c r="D459" s="44" t="s">
-        <v>722</v>
+        <v>717</v>
+      </c>
+      <c r="D459" s="45" t="s">
+        <v>718</v>
       </c>
       <c r="E459" s="43"/>
       <c r="F459" s="44"/>
@@ -8805,8 +8852,12 @@
     <row r="460" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A460" s="43"/>
       <c r="B460" s="44"/>
-      <c r="C460" s="43"/>
-      <c r="D460" s="44"/>
+      <c r="C460" s="43" t="s">
+        <v>728</v>
+      </c>
+      <c r="D460" s="44" t="s">
+        <v>729</v>
+      </c>
       <c r="E460" s="43"/>
       <c r="F460" s="44"/>
       <c r="G460" s="44"/>
@@ -8814,6 +8865,85 @@
       <c r="I460" s="44"/>
       <c r="J460" s="44"/>
       <c r="K460" s="44"/>
+    </row>
+    <row r="461" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A461" s="43"/>
+      <c r="B461" s="44"/>
+      <c r="C461" s="43" t="s">
+        <v>719</v>
+      </c>
+      <c r="D461" s="44"/>
+      <c r="E461" s="43"/>
+      <c r="F461" s="44"/>
+      <c r="G461" s="44"/>
+      <c r="H461" s="44"/>
+      <c r="I461" s="44"/>
+      <c r="J461" s="44"/>
+      <c r="K461" s="44"/>
+    </row>
+    <row r="462" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A462" s="43"/>
+      <c r="B462" s="44"/>
+      <c r="C462" s="43" t="s">
+        <v>720</v>
+      </c>
+      <c r="D462" s="44" t="s">
+        <v>723</v>
+      </c>
+      <c r="E462" s="43"/>
+      <c r="F462" s="44"/>
+      <c r="G462" s="44"/>
+      <c r="H462" s="44"/>
+      <c r="I462" s="44"/>
+      <c r="J462" s="44"/>
+      <c r="K462" s="44"/>
+    </row>
+    <row r="463" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A463" s="43"/>
+      <c r="B463" s="44"/>
+      <c r="C463" s="43" t="s">
+        <v>725</v>
+      </c>
+      <c r="D463" s="44" t="s">
+        <v>724</v>
+      </c>
+      <c r="E463" s="43"/>
+      <c r="F463" s="44"/>
+      <c r="G463" s="44"/>
+      <c r="H463" s="44"/>
+      <c r="I463" s="44"/>
+      <c r="J463" s="44"/>
+      <c r="K463" s="44"/>
+    </row>
+    <row r="464" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A464" s="43"/>
+      <c r="B464" s="44"/>
+      <c r="C464" s="43" t="s">
+        <v>721</v>
+      </c>
+      <c r="D464" s="44" t="s">
+        <v>722</v>
+      </c>
+      <c r="E464" s="43"/>
+      <c r="F464" s="44"/>
+      <c r="G464" s="44"/>
+      <c r="H464" s="44"/>
+      <c r="I464" s="44"/>
+      <c r="J464" s="44"/>
+      <c r="K464" s="44"/>
+    </row>
+    <row r="465" spans="1:11" x14ac:dyDescent="0.35">
+      <c r="A465" s="43"/>
+      <c r="B465" s="44"/>
+      <c r="C465" s="43"/>
+      <c r="D465" s="44"/>
+      <c r="E465" s="43"/>
+      <c r="F465" s="44"/>
+      <c r="G465" s="44"/>
+      <c r="H465" s="44"/>
+      <c r="I465" s="44"/>
+      <c r="J465" s="44"/>
+      <c r="K465" s="44"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>

</xml_diff>